<commit_message>
Add annotation short to Oligo notes table
</commit_message>
<xml_diff>
--- a/processed-data/19_other_Oligo/00_check_Oligo_markers/ERC_Oligo_notes.xlsx
+++ b/processed-data/19_other_Oligo/00_check_Oligo_markers/ERC_Oligo_notes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lieberinstitute-my.sharepoint.com/personal/louise_huuki_libd_org/Documents/LIBD_code/LFF_spatial_ERC/processed-data/19_other_Oligo/00_check_Oligo_markers/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="13_ncr:1_{45DC2D14-E444-3940-B2F7-9E131A33B774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CABC204F-7EA9-F945-9022-D013B298D950}"/>
+  <xr:revisionPtr revIDLastSave="40" documentId="13_ncr:1_{45DC2D14-E444-3940-B2F7-9E131A33B774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E80A66AE-3A5B-724E-ABEB-E4A05E451D84}"/>
   <bookViews>
-    <workbookView xWindow="640" yWindow="760" windowWidth="28540" windowHeight="17400" activeTab="1" xr2:uid="{D3C45F6A-23E9-DF44-BEE0-E5DD3B4BB180}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17800" xr2:uid="{D3C45F6A-23E9-DF44-BEE0-E5DD3B4BB180}"/>
   </bookViews>
   <sheets>
     <sheet name="Oligo Annotations" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="146">
   <si>
     <t>OPC</t>
   </si>
@@ -500,6 +500,27 @@
   </si>
   <si>
     <t>check markers</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1016/j.neuron.2024.11.016</t>
+  </si>
+  <si>
+    <t>DOI</t>
+  </si>
+  <si>
+    <t>Annotation_short</t>
+  </si>
+  <si>
+    <t>Oligo.NF</t>
+  </si>
+  <si>
+    <t>Oligo.M</t>
+  </si>
+  <si>
+    <t>Oligo.L</t>
+  </si>
+  <si>
+    <t>Oligo.P</t>
   </si>
 </sst>
 </file>
@@ -629,6 +650,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -948,21 +973,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8118FE2-0B82-7D4D-BDF4-7C654142C9BA}">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.6640625" style="3" customWidth="1"/>
-    <col min="2" max="2" width="15.6640625" style="3" customWidth="1"/>
-    <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.6640625" customWidth="1"/>
+    <col min="2" max="3" width="15.6640625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="15" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="52" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>136</v>
       </c>
@@ -970,49 +995,52 @@
         <v>41</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="2">
+        <v>0</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="1"/>
+      <c r="G2" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>21</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>21</v>
@@ -1021,164 +1049,182 @@
         <v>21</v>
       </c>
       <c r="J2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="K2" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="51" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="D3" s="2">
         <v>1</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="F3" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="J3" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="K3" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="D4" s="2">
         <v>2</v>
       </c>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="1"/>
+      <c r="F4" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="I4" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="J4" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="K4" s="1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D5" s="2">
         <v>3</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="I5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="J5" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="K5" s="1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D6" s="2">
         <v>4</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="I6" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="J6" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="K6" s="1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>2</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="D7" s="2">
         <v>5</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="H7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="I7" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="J7" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="K7" s="1" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1191,7 +1237,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A010F79-2158-CA4E-B969-AC78B6395658}">
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="28.83203125" bestFit="1" customWidth="1"/>
@@ -1200,15 +1246,16 @@
     <col min="4" max="4" width="58" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20.1640625" customWidth="1"/>
     <col min="6" max="6" width="27.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="54.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.1640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="35.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="38.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="54.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.1640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="35.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" s="7" t="s">
         <v>45</v>
       </c>
@@ -1228,25 +1275,28 @@
         <v>48</v>
       </c>
       <c r="G1" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="H1" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="I1" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="J1" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="K1" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="L1" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="L1" s="7" t="s">
+      <c r="M1" s="7" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
         <v>50</v>
       </c>
@@ -1261,15 +1311,16 @@
       <c r="F2" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3" t="b">
+      <c r="G2" s="6"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="J2" s="3" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>54</v>
       </c>
@@ -1288,26 +1339,27 @@
       <c r="F3" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="6"/>
+      <c r="H3" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="H3" s="3" t="b">
+      <c r="I3" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="J3" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="K3" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="L3" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="M3" s="3" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
         <v>58</v>
       </c>
@@ -1326,18 +1378,19 @@
       <c r="F4" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="6"/>
+      <c r="H4" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H4" s="3" t="b">
+      <c r="I4" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="I4" s="3"/>
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
       <c r="L4" s="3"/>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M4" s="3"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
         <v>63</v>
       </c>
@@ -1354,26 +1407,27 @@
       <c r="F5" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G5" s="6"/>
+      <c r="H5" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="H5" s="3" t="b">
+      <c r="I5" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="J5" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="J5" s="6" t="s">
+      <c r="K5" s="6" t="s">
         <v>108</v>
-      </c>
-      <c r="K5" s="6" t="s">
-        <v>109</v>
       </c>
       <c r="L5" s="6" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M5" s="6" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
         <v>79</v>
       </c>
@@ -1386,26 +1440,27 @@
       </c>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
-      <c r="G6" s="6" t="s">
+      <c r="G6" s="6"/>
+      <c r="H6" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="I6" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="I6" s="6" t="s">
+      <c r="J6" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="J6" s="6" t="s">
+      <c r="K6" s="6" t="s">
         <v>110</v>
-      </c>
-      <c r="K6" s="6" t="s">
-        <v>112</v>
       </c>
       <c r="L6" s="6" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M6" s="6" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
         <v>65</v>
       </c>
@@ -1424,26 +1479,27 @@
       <c r="F7" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="G7" s="6"/>
+      <c r="H7" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="H7" s="3" t="b">
+      <c r="I7" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="I7" s="6" t="s">
+      <c r="J7" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="J7" s="3" t="s">
+      <c r="K7" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="K7" s="3" t="s">
+      <c r="L7" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="L7" s="3" t="s">
+      <c r="M7" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
         <v>92</v>
       </c>
@@ -1462,26 +1518,27 @@
       <c r="F8" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="G8" s="6"/>
+      <c r="H8" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="H8" s="3" t="b">
+      <c r="I8" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="I8" s="3" t="s">
+      <c r="J8" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="J8" s="3" t="s">
+      <c r="K8" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="K8" s="3" t="s">
+      <c r="L8" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="L8" s="3" t="s">
+      <c r="M8" s="3" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
         <v>71</v>
       </c>
@@ -1500,26 +1557,27 @@
       <c r="F9" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="G9" s="6"/>
+      <c r="H9" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="H9" s="3" t="b">
+      <c r="I9" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="I9" s="3" t="s">
+      <c r="J9" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="J9" s="3" t="s">
+      <c r="K9" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="K9" s="3" t="s">
+      <c r="L9" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="L9" s="3" t="s">
+      <c r="M9" s="3" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
         <v>74</v>
       </c>
@@ -1538,26 +1596,27 @@
       <c r="F10" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="G10" s="3"/>
+      <c r="H10" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="H10" s="3" t="b">
+      <c r="I10" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="I10" s="3" t="s">
+      <c r="J10" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="J10" s="3" t="s">
+      <c r="K10" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="K10" s="3" t="s">
+      <c r="L10" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="L10" s="3" t="s">
+      <c r="M10" s="3" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
         <v>128</v>
       </c>
@@ -1573,33 +1632,36 @@
       <c r="E11" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="G11" s="6" t="s">
+      <c r="G11" t="s">
+        <v>139</v>
+      </c>
+      <c r="H11" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="H11" s="3" t="b">
+      <c r="I11" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="I11" s="3" t="s">
+      <c r="J11" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="J11" s="3" t="s">
+      <c r="K11" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="K11" s="3" t="s">
+      <c r="L11" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="L11" s="3" t="s">
+      <c r="M11" s="3" t="s">
         <v>133</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="H2:H11">
+  <conditionalFormatting sqref="I2:I11">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
-      <formula>$H$3</formula>
+      <formula>$I$3</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
-      <formula>$H$3</formula>
+      <formula>$I$3</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update Oligo.4 annotation to pre-myelinating
</commit_message>
<xml_diff>
--- a/processed-data/19_other_Oligo/00_check_Oligo_markers/ERC_Oligo_notes.xlsx
+++ b/processed-data/19_other_Oligo/00_check_Oligo_markers/ERC_Oligo_notes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lieberinstitute-my.sharepoint.com/personal/louise_huuki_libd_org/Documents/LIBD_code/LFF_spatial_ERC/processed-data/19_other_Oligo/00_check_Oligo_markers/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="48" documentId="13_ncr:1_{45DC2D14-E444-3940-B2F7-9E131A33B774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A1635038-D87A-DB4B-80EF-B5A95C4CCB6C}"/>
+  <xr:revisionPtr revIDLastSave="52" documentId="13_ncr:1_{45DC2D14-E444-3940-B2F7-9E131A33B774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{421F8BEA-9673-434A-9427-D6525E516265}"/>
   <bookViews>
-    <workbookView xWindow="44520" yWindow="1720" windowWidth="30240" windowHeight="17800" xr2:uid="{D3C45F6A-23E9-DF44-BEE0-E5DD3B4BB180}"/>
+    <workbookView xWindow="38400" yWindow="1720" windowWidth="30240" windowHeight="17800" xr2:uid="{D3C45F6A-23E9-DF44-BEE0-E5DD3B4BB180}"/>
   </bookViews>
   <sheets>
     <sheet name="Oligo Annotations" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="148">
   <si>
     <t>OPC</t>
   </si>
@@ -520,7 +520,13 @@
     <t>Oligo.L</t>
   </si>
   <si>
-    <t>Oligo.P</t>
+    <t>Oligo.PM</t>
+  </si>
+  <si>
+    <t>Oligo.PV</t>
+  </si>
+  <si>
+    <t>Pre-myelinating Oligo</t>
   </si>
 </sst>
 </file>
@@ -650,10 +656,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -977,7 +979,8 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.6640625" style="3" customWidth="1"/>
-    <col min="2" max="3" width="15.6640625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="18.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.6640625" style="3" customWidth="1"/>
     <col min="4" max="4" width="15" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7.5" bestFit="1" customWidth="1"/>
@@ -1106,7 +1109,7 @@
         <v>124</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D4" s="2">
         <v>2</v>
@@ -1139,10 +1142,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>127</v>
+        <v>147</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D5" s="2">
         <v>3</v>

</xml_diff>